<commit_message>
new data check on dollarization and unused credit
</commit_message>
<xml_diff>
--- a/data/documentation/dictionary_muestra_anonima_base2015.xlsx
+++ b/data/documentation/dictionary_muestra_anonima_base2015.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/guilhermeluz/Desktop/Credit_lines_Peru/data/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DDD65B9-AB1B-8444-A3D6-3A220DB02FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26AE9814-9A18-3F47-B032-2F68B7D3A425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4787" uniqueCount="1037">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4784" uniqueCount="1034">
   <si>
     <t>Data dictionary - muestra_anonima_base2015.parquet</t>
   </si>
@@ -3057,15 +3057,6 @@
   </si>
   <si>
     <t>context</t>
-  </si>
-  <si>
-    <t>Balance units</t>
-  </si>
-  <si>
-    <t>Are the credito_* / linea_* balances in soles for every row (foreign-currency balances converted), or in the original currency of moneda_codigo? Which scale (units, thousands)?</t>
-  </si>
-  <si>
-    <t>The RCC dictionary has no currency field, and the data cannot settle it. It matters for any cross-currency aggregation. Also: one row (entidad 365, 2010-09-30, corporativo / arrendamiento_financiero) has credito_utilizado = 294,880,000,000, about 70x the next-largest value; it looks like an error.</t>
   </si>
   <si>
     <t>moneda_codigo = 3</t>
@@ -3630,7 +3621,7 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
     </row>
   </sheetData>
@@ -24831,81 +24822,75 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="42" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>1008</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1009</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>1010</v>
-      </c>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" ht="28" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>1011</v>
+        <v>1008</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1012</v>
+        <v>1009</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>1013</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="28" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1015</v>
+        <v>1012</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>1016</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>1018</v>
+        <v>1015</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>1019</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>1020</v>
+        <v>1017</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>1021</v>
+        <v>1018</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="28" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>1023</v>
+        <v>1020</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>1024</v>
+        <v>1021</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>1025</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="42" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>1026</v>
+        <v>1023</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>1027</v>
+        <v>1024</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>1028</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="28" x14ac:dyDescent="0.2">
@@ -24913,10 +24898,10 @@
         <v>201</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>1029</v>
+        <v>1026</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>1030</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -24924,21 +24909,21 @@
         <v>125</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>1031</v>
+        <v>1028</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>1032</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>1035</v>
+        <v>1032</v>
       </c>
     </row>
   </sheetData>

</xml_diff>